<commit_message>
feat: add morning/evening report types, snapshot rotation, and toggle buttons in report pages
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="18 Juli" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 Juli" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
feat: tambah target harian dan pewarnaan kondisional di Excel report
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="18 Juli" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 Juli" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data: 22 Juli 2026 pukul 09.35 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="21 Juli" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22 Juli" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data: 24 Juli 2026 pukul 11.14 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="24 Juli" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24 Juli" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data: 25 Juli 2026 pukul 11.53 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="25 Juli" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25 Juli" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
feat: tambahkan pewarnaan progres harian dan nama kecamatan pada report monitoring dan excel
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1 Juli" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Juli" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data: 9 Agustus 2026 pukul 11.00 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="9 Agustus" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Agustus" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data: 10 Agustus 2026 pukul 21.10 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="10 Agustus" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Agustus" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data: 15 Agustus 2026 pukul 09.28 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Latest.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="13 Agustus" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Agustus" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>